<commit_message>
Rewrite PDF generator with ReportLab for clean aligned layout
Replace fpdf2 (cursor bugs caused cutoff text fragments on the right margin)
with ReportLab Platypus flow layout: equal margins, section header bars,
two-column summary table, and proper bullet lists with no off-center text.

Co-authored-by: vengeanceaiUSC <vengeanceaiUSC@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/.cursor/skills/syllabus-dissector/example_output/documents/syllabi.xlsx
+++ b/.cursor/skills/syllabus-dissector/example_output/documents/syllabi.xlsx
@@ -95,7 +95,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -116,6 +116,18 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -641,27 +653,27 @@
           <t>Sleep Paper</t>
         </is>
       </c>
-      <c r="B8" s="23" t="inlineStr">
+      <c r="B8" s="27" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
       </c>
-      <c r="C8" s="23" t="inlineStr">
+      <c r="C8" s="27" t="inlineStr">
         <is>
           <t>2025-09-04</t>
         </is>
       </c>
-      <c r="D8" s="23" t="inlineStr">
+      <c r="D8" s="27" t="inlineStr">
         <is>
           <t>2025-09-15</t>
         </is>
       </c>
-      <c r="E8" s="23" t="inlineStr">
+      <c r="E8" s="27" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F8" s="24">
+      <c r="F8" s="28">
         <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/hist-103-sleep-paper.pdf","Open PDF")</f>
         <v/>
       </c>
@@ -672,27 +684,27 @@
           <t>Witchcraft Paper</t>
         </is>
       </c>
-      <c r="B9" s="25" t="inlineStr">
+      <c r="B9" s="29" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
       </c>
-      <c r="C9" s="25" t="inlineStr">
+      <c r="C9" s="29" t="inlineStr">
         <is>
           <t>2025-11-06</t>
         </is>
       </c>
-      <c r="D9" s="25" t="inlineStr">
+      <c r="D9" s="29" t="inlineStr">
         <is>
           <t>2025-11-10</t>
         </is>
       </c>
-      <c r="E9" s="25" t="inlineStr">
+      <c r="E9" s="29" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F9" s="26">
+      <c r="F9" s="30">
         <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/hist-103-witchcraft-paper.pdf","Open PDF")</f>
         <v/>
       </c>
@@ -703,27 +715,27 @@
           <t>Mid-term</t>
         </is>
       </c>
-      <c r="B10" s="23" t="inlineStr">
+      <c r="B10" s="27" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
       </c>
-      <c r="C10" s="23" t="inlineStr">
+      <c r="C10" s="27" t="inlineStr">
         <is>
           <t>2025-08-25</t>
         </is>
       </c>
-      <c r="D10" s="23" t="inlineStr">
+      <c r="D10" s="27" t="inlineStr">
         <is>
           <t>2025-10-06</t>
         </is>
       </c>
-      <c r="E10" s="23" t="inlineStr">
+      <c r="E10" s="27" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F10" s="24">
+      <c r="F10" s="28">
         <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/hist-103-mid-term.pdf","Open PDF")</f>
         <v/>
       </c>
@@ -734,27 +746,27 @@
           <t>Final Exam</t>
         </is>
       </c>
-      <c r="B11" s="25" t="inlineStr">
+      <c r="B11" s="29" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
       </c>
-      <c r="C11" s="25" t="inlineStr">
+      <c r="C11" s="29" t="inlineStr">
         <is>
           <t>2025-10-13</t>
         </is>
       </c>
-      <c r="D11" s="25" t="inlineStr">
+      <c r="D11" s="29" t="inlineStr">
         <is>
           <t>2025-12-10</t>
         </is>
       </c>
-      <c r="E11" s="25" t="inlineStr">
+      <c r="E11" s="29" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F11" s="26">
+      <c r="F11" s="30">
         <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/hist-103-final-exam.pdf","Open PDF")</f>
         <v/>
       </c>
@@ -765,27 +777,27 @@
           <t>Discussion Section</t>
         </is>
       </c>
-      <c r="B12" s="23" t="inlineStr">
+      <c r="B12" s="27" t="inlineStr">
         <is>
           <t>15%</t>
         </is>
       </c>
-      <c r="C12" s="23" t="inlineStr">
+      <c r="C12" s="27" t="inlineStr">
         <is>
           <t>2025-08-25</t>
         </is>
       </c>
-      <c r="D12" s="23" t="inlineStr">
+      <c r="D12" s="27" t="inlineStr">
         <is>
           <t>2025-12-04</t>
         </is>
       </c>
-      <c r="E12" s="23" t="inlineStr">
+      <c r="E12" s="27" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F12" s="24">
+      <c r="F12" s="28">
         <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/hist-103-discussion-section.pdf","Open PDF")</f>
         <v/>
       </c>
@@ -796,27 +808,27 @@
           <t>Identification Quizzes</t>
         </is>
       </c>
-      <c r="B13" s="25" t="inlineStr">
+      <c r="B13" s="29" t="inlineStr">
         <is>
           <t>5%</t>
         </is>
       </c>
-      <c r="C13" s="25" t="inlineStr">
+      <c r="C13" s="29" t="inlineStr">
         <is>
           <t>2025-08-25</t>
         </is>
       </c>
-      <c r="D13" s="25" t="inlineStr">
+      <c r="D13" s="29" t="inlineStr">
         <is>
           <t>2025-12-03</t>
         </is>
       </c>
-      <c r="E13" s="25" t="inlineStr">
+      <c r="E13" s="29" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F13" s="26">
+      <c r="F13" s="30">
         <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/hist-103-identification-quizzes.pdf","Open PDF")</f>
         <v/>
       </c>
@@ -827,27 +839,27 @@
           <t>Extra Credit</t>
         </is>
       </c>
-      <c r="B14" s="23" t="inlineStr">
+      <c r="B14" s="27" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="C14" s="23" t="inlineStr">
+      <c r="C14" s="27" t="inlineStr">
         <is>
           <t>2025-08-25</t>
         </is>
       </c>
-      <c r="D14" s="23" t="inlineStr">
+      <c r="D14" s="27" t="inlineStr">
         <is>
           <t>2025-12-04</t>
         </is>
       </c>
-      <c r="E14" s="23" t="inlineStr">
+      <c r="E14" s="27" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F14" s="24">
+      <c r="F14" s="28">
         <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/hist-103-extra-credit.pdf","Open PDF")</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Add automatic full-syllabus grep via auto_dissect.py
Replace manual JSON authoring with auto_dissect.py that detects categories
from the Assignments section, greps every paragraph in the full syllabus,
captures dedicated assignment blocks (prompts, study guides, extra credit),
structures sections, and archives verbatim text. Add dissect_syllabus.py
one-command pipeline; update SKILL.md and reference.md.

Co-authored-by: vengeanceaiUSC <vengeanceaiUSC@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/.cursor/skills/syllabus-dissector/example_output/documents/syllabi.xlsx
+++ b/.cursor/skills/syllabus-dissector/example_output/documents/syllabi.xlsx
@@ -95,7 +95,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -116,6 +116,30 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -611,7 +635,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>A: 100-93; A-: 92-90; B+: 89-87; B: 86-83; B-: 82-80; C+: 79-77; C: 76-73; C-: 72-70; D+: 69-67; D: 66-63; D-: 62-60; F: 59-0</t>
+          <t>A: 100-93; A-: 92-90; B+: 89-87; B: 86-83; B-: 82-80; C+: 79-77; C: 76-73; C- 72-70 D+: 69-67; D: 66-63; D-: 62-60; F: 59-0</t>
         </is>
       </c>
     </row>
@@ -653,27 +677,27 @@
           <t>Sleep Paper</t>
         </is>
       </c>
-      <c r="B8" s="27" t="inlineStr">
+      <c r="B8" s="35" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
       </c>
-      <c r="C8" s="27" t="inlineStr">
-        <is>
-          <t>2025-09-04</t>
-        </is>
-      </c>
-      <c r="D8" s="27" t="inlineStr">
-        <is>
-          <t>2025-09-15</t>
-        </is>
-      </c>
-      <c r="E8" s="27" t="inlineStr">
+      <c r="C8" s="35" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="D8" s="35" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="E8" s="35" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F8" s="28">
+      <c r="F8" s="36">
         <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/hist-103-sleep-paper.pdf","Open PDF")</f>
         <v/>
       </c>
@@ -684,27 +708,27 @@
           <t>Witchcraft Paper</t>
         </is>
       </c>
-      <c r="B9" s="29" t="inlineStr">
+      <c r="B9" s="37" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
       </c>
-      <c r="C9" s="29" t="inlineStr">
-        <is>
-          <t>2025-11-06</t>
-        </is>
-      </c>
-      <c r="D9" s="29" t="inlineStr">
-        <is>
-          <t>2025-11-10</t>
-        </is>
-      </c>
-      <c r="E9" s="29" t="inlineStr">
+      <c r="C9" s="37" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="D9" s="37" t="inlineStr">
+        <is>
+          <t>2026-11-10</t>
+        </is>
+      </c>
+      <c r="E9" s="37" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F9" s="30">
+      <c r="F9" s="38">
         <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/hist-103-witchcraft-paper.pdf","Open PDF")</f>
         <v/>
       </c>
@@ -715,27 +739,27 @@
           <t>Mid-term</t>
         </is>
       </c>
-      <c r="B10" s="27" t="inlineStr">
+      <c r="B10" s="35" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
       </c>
-      <c r="C10" s="27" t="inlineStr">
-        <is>
-          <t>2025-08-25</t>
-        </is>
-      </c>
-      <c r="D10" s="27" t="inlineStr">
-        <is>
-          <t>2025-10-06</t>
-        </is>
-      </c>
-      <c r="E10" s="27" t="inlineStr">
+      <c r="C10" s="35" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="D10" s="35" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="E10" s="35" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F10" s="28">
+      <c r="F10" s="36">
         <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/hist-103-mid-term.pdf","Open PDF")</f>
         <v/>
       </c>
@@ -746,27 +770,27 @@
           <t>Final Exam</t>
         </is>
       </c>
-      <c r="B11" s="29" t="inlineStr">
+      <c r="B11" s="37" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
       </c>
-      <c r="C11" s="29" t="inlineStr">
-        <is>
-          <t>2025-10-13</t>
-        </is>
-      </c>
-      <c r="D11" s="29" t="inlineStr">
-        <is>
-          <t>2025-12-10</t>
-        </is>
-      </c>
-      <c r="E11" s="29" t="inlineStr">
+      <c r="C11" s="37" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="D11" s="37" t="inlineStr">
+        <is>
+          <t>2026-12-10</t>
+        </is>
+      </c>
+      <c r="E11" s="37" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F11" s="30">
+      <c r="F11" s="38">
         <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/hist-103-final-exam.pdf","Open PDF")</f>
         <v/>
       </c>
@@ -777,27 +801,27 @@
           <t>Discussion Section</t>
         </is>
       </c>
-      <c r="B12" s="27" t="inlineStr">
+      <c r="B12" s="35" t="inlineStr">
         <is>
           <t>15%</t>
         </is>
       </c>
-      <c r="C12" s="27" t="inlineStr">
-        <is>
-          <t>2025-08-25</t>
-        </is>
-      </c>
-      <c r="D12" s="27" t="inlineStr">
-        <is>
-          <t>2025-12-04</t>
-        </is>
-      </c>
-      <c r="E12" s="27" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F12" s="28">
+      <c r="C12" s="35" t="inlineStr">
+        <is>
+          <t>2026-11-10</t>
+        </is>
+      </c>
+      <c r="D12" s="35" t="inlineStr">
+        <is>
+          <t>2026-11-12</t>
+        </is>
+      </c>
+      <c r="E12" s="35" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F12" s="36">
         <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/hist-103-discussion-section.pdf","Open PDF")</f>
         <v/>
       </c>
@@ -808,27 +832,27 @@
           <t>Identification Quizzes</t>
         </is>
       </c>
-      <c r="B13" s="29" t="inlineStr">
+      <c r="B13" s="37" t="inlineStr">
         <is>
           <t>5%</t>
         </is>
       </c>
-      <c r="C13" s="29" t="inlineStr">
-        <is>
-          <t>2025-08-25</t>
-        </is>
-      </c>
-      <c r="D13" s="29" t="inlineStr">
-        <is>
-          <t>2025-12-03</t>
-        </is>
-      </c>
-      <c r="E13" s="29" t="inlineStr">
+      <c r="C13" s="37" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="D13" s="37" t="inlineStr">
+        <is>
+          <t>2026-12-10</t>
+        </is>
+      </c>
+      <c r="E13" s="37" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F13" s="30">
+      <c r="F13" s="38">
         <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/hist-103-identification-quizzes.pdf","Open PDF")</f>
         <v/>
       </c>
@@ -839,27 +863,23 @@
           <t>Extra Credit</t>
         </is>
       </c>
-      <c r="B14" s="27" t="inlineStr">
+      <c r="B14" s="35" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="C14" s="27" t="inlineStr">
-        <is>
-          <t>2025-08-25</t>
-        </is>
-      </c>
-      <c r="D14" s="27" t="inlineStr">
-        <is>
-          <t>2025-12-04</t>
-        </is>
-      </c>
-      <c r="E14" s="27" t="inlineStr">
+      <c r="C14" s="35" t="inlineStr"/>
+      <c r="D14" s="35" t="inlineStr">
+        <is>
+          <t>2026-12-04</t>
+        </is>
+      </c>
+      <c r="E14" s="35" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F14" s="28">
+      <c r="F14" s="36">
         <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/hist-103-extra-credit.pdf","Open PDF")</f>
         <v/>
       </c>

</xml_diff>